<commit_message>
docs: add PN532 NFC module to BOM
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Co-authored-by: multica-agent <github@multica.ai>
</commit_message>
<xml_diff>
--- a/STM32U5_BOM.xlsx
+++ b/STM32U5_BOM.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -763,7 +763,7 @@
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>三、告警输出</t>
+          <t>三、通信模块</t>
         </is>
       </c>
       <c r="B10" s="10" t="n"/>
@@ -781,12 +781,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>微型振动马达</t>
+          <t>NFC 读写模块</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>1027 扁平偏心轮电机</t>
+          <t>PN532 NFC RFID V3 模块</t>
         </is>
       </c>
       <c r="D11" s="11" t="n">
@@ -799,203 +799,203 @@
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
+          <t>C232619</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>¥18</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>13.56MHz NFC 读写/卡模拟，I2C/SPI/UART</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>搜索"PN532模块"，支持 NTAG/NFC Tag/Mifare</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>四、告警输出</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="10" t="n"/>
+      <c r="H12" s="10" t="n"/>
+      <c r="I12" s="10" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>微型振动马达</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>1027 扁平偏心轮电机</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
           <t>C2895556</t>
         </is>
       </c>
-      <c r="G11" s="12" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>¥3</t>
         </is>
       </c>
-      <c r="H11" s="12" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>跌倒/倾斜触觉告警，PWM 调速</t>
         </is>
       </c>
-      <c r="I11" s="12" t="inlineStr">
+      <c r="I13" s="7" t="inlineStr">
         <is>
           <t>需配 NPN 三极管驱动 (如 S8050 C2146)</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>NPN 三极管</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>S8050 (TO-92)</t>
         </is>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D14" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E14" s="13" t="inlineStr">
         <is>
           <t>个</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F14" s="11" t="inlineStr">
         <is>
           <t>C2146</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G14" s="12" t="inlineStr">
         <is>
           <t>¥0.2</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H14" s="12" t="inlineStr">
         <is>
           <t>驱动振动马达</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr"/>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="I14" s="12" t="inlineStr"/>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>直插 RGB LED 共阴</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>5mm 共阴三色 LED</t>
         </is>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D15" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>个</t>
         </is>
       </c>
-      <c r="F13" s="11" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>C965027</t>
         </is>
       </c>
-      <c r="G13" s="12" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>¥1</t>
         </is>
       </c>
-      <c r="H13" s="12" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>状态指示: 绿(正常) 黄(倾斜) 红(跌倒)</t>
         </is>
       </c>
-      <c r="I13" s="12" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>需 3 颗 220Ω 限流电阻</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>直插电阻 220Ω</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>1/4W ±5% 碳膜</t>
         </is>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D16" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E16" s="13" t="inlineStr">
         <is>
           <t>个</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F16" s="11" t="inlineStr">
         <is>
           <t>C17405</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G16" s="12" t="inlineStr">
         <is>
           <t>¥0.1</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H16" s="12" t="inlineStr">
         <is>
           <t>RGB LED 限流</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr"/>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>有源蜂鸣器模块 (可选)</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>3.3V 有源蜂鸣器</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="13" t="inlineStr">
-        <is>
-          <t>个</t>
-        </is>
-      </c>
-      <c r="F15" s="11" t="inlineStr">
-        <is>
-          <t>C31955</t>
-        </is>
-      </c>
-      <c r="G15" s="12" t="inlineStr">
-        <is>
-          <t>¥2</t>
-        </is>
-      </c>
-      <c r="H15" s="12" t="inlineStr">
-        <is>
-          <t>声音告警辅助</t>
-        </is>
-      </c>
-      <c r="I15" s="12" t="inlineStr">
-        <is>
-          <t>搜索"3.3V有源蜂鸣器模块"</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
-        <is>
-          <t>四、输入交互</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
-      <c r="H16" s="10" t="n"/>
-      <c r="I16" s="10" t="n"/>
+      <c r="I16" s="12" t="inlineStr"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -1003,96 +1003,100 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
+          <t>有源蜂鸣器模块 (可选)</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>3.3V 有源蜂鸣器</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>C31955</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>¥2</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>声音告警辅助</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>搜索"3.3V有源蜂鸣器模块"</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>五、输入交互</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="n"/>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="10" t="n"/>
+      <c r="E18" s="10" t="n"/>
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="10" t="n"/>
+      <c r="H18" s="10" t="n"/>
+      <c r="I18" s="10" t="n"/>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
           <t>轻触开关 6x6mm</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>6x6x5mm 四脚轻触</t>
         </is>
       </c>
-      <c r="D17" s="6" t="n">
+      <c r="D19" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E19" s="13" t="inlineStr">
         <is>
           <t>个</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F19" s="11" t="inlineStr">
         <is>
           <t>C31892</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G19" s="12" t="inlineStr">
         <is>
           <t>¥0.3</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H19" s="12" t="inlineStr">
         <is>
           <t>长按解除告警 + 预留功能按键</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="I19" s="12" t="inlineStr">
         <is>
           <t>配 10kΩ 上拉电阻</t>
         </is>
       </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>直插电阻 10kΩ</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>1/4W ±5% 碳膜</t>
-        </is>
-      </c>
-      <c r="D18" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E18" s="13" t="inlineStr">
-        <is>
-          <t>个</t>
-        </is>
-      </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>C17408</t>
-        </is>
-      </c>
-      <c r="G18" s="12" t="inlineStr">
-        <is>
-          <t>¥0.1</t>
-        </is>
-      </c>
-      <c r="H18" s="12" t="inlineStr">
-        <is>
-          <t>按键上拉</t>
-        </is>
-      </c>
-      <c r="I18" s="12" t="inlineStr"/>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>五、电源系统</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="n"/>
-      <c r="C19" s="10" t="n"/>
-      <c r="D19" s="10" t="n"/>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
-      <c r="H19" s="10" t="n"/>
-      <c r="I19" s="10" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="6" t="n">
@@ -1100,143 +1104,139 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
+          <t>直插电阻 10kΩ</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>1/4W ±5% 碳膜</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>C17408</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>¥0.1</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>按键上拉</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>六、电源系统</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="n"/>
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="10" t="n"/>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="10" t="n"/>
+      <c r="H21" s="10" t="n"/>
+      <c r="I21" s="10" t="n"/>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
           <t>AMS1117-3.3V 稳压模块</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>AMS1117-3.3 降压模块</t>
         </is>
       </c>
-      <c r="D20" s="6" t="n">
+      <c r="D22" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E20" s="8" t="inlineStr">
+      <c r="E22" s="13" t="inlineStr">
         <is>
           <t>个</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F22" s="11" t="inlineStr">
         <is>
           <t>C6186</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G22" s="12" t="inlineStr">
         <is>
           <t>¥2</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H22" s="12" t="inlineStr">
         <is>
           <t>电池 3.7V → 3.3V 稳定供电</t>
         </is>
       </c>
-      <c r="I20" s="7" t="inlineStr">
+      <c r="I22" s="12" t="inlineStr">
         <is>
           <t>或直接用 NUCLEO Vin 引脚 (5V)</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="11" t="n">
-        <v>12</v>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>TP4056 锂电池充电模块</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>TP4056 Type-C 充电板</t>
         </is>
       </c>
-      <c r="D21" s="11" t="n">
+      <c r="D23" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="13" t="inlineStr">
+      <c r="E23" s="8" t="inlineStr">
         <is>
           <t>个</t>
         </is>
       </c>
-      <c r="F21" s="11" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>C382139</t>
         </is>
       </c>
-      <c r="G21" s="12" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>¥3</t>
         </is>
       </c>
-      <c r="H21" s="12" t="inlineStr">
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>锂电池充电管理，含过充过放保护</t>
         </is>
       </c>
-      <c r="I21" s="12" t="inlineStr">
+      <c r="I23" s="7" t="inlineStr">
         <is>
           <t>搜索"TP4056充电模块 Type-C"</t>
         </is>
       </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>锂聚合物电池</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>3.7V 800mAh 502535</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>块</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>¥15</t>
-        </is>
-      </c>
-      <c r="H22" s="7" t="inlineStr">
-        <is>
-          <t>可穿戴独立供电</t>
-        </is>
-      </c>
-      <c r="I22" s="7" t="inlineStr">
-        <is>
-          <t>淘宝购买，立创不售电池</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>六、连接与固定</t>
-        </is>
-      </c>
-      <c r="B23" s="10" t="n"/>
-      <c r="C23" s="10" t="n"/>
-      <c r="D23" s="10" t="n"/>
-      <c r="E23" s="10" t="n"/>
-      <c r="F23" s="10" t="n"/>
-      <c r="G23" s="10" t="n"/>
-      <c r="H23" s="10" t="n"/>
-      <c r="I23" s="10" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="11" t="n">
@@ -1244,12 +1244,12 @@
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>杜邦线 母对母 20cm</t>
+          <t>锂聚合物电池</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>2.54mm 1P-1P 20cm</t>
+          <t>3.7V 800mAh 502535</t>
         </is>
       </c>
       <c r="D24" s="11" t="n">
@@ -1257,257 +1257,285 @@
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
+          <t>块</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>¥15</t>
+        </is>
+      </c>
+      <c r="H24" s="12" t="inlineStr">
+        <is>
+          <t>可穿戴独立供电</t>
+        </is>
+      </c>
+      <c r="I24" s="12" t="inlineStr">
+        <is>
+          <t>淘宝购买，立创不售电池</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>七、连接与固定</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="n"/>
+      <c r="C25" s="10" t="n"/>
+      <c r="D25" s="10" t="n"/>
+      <c r="E25" s="10" t="n"/>
+      <c r="F25" s="10" t="n"/>
+      <c r="G25" s="10" t="n"/>
+      <c r="H25" s="10" t="n"/>
+      <c r="I25" s="10" t="n"/>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>杜邦线 母对母 20cm</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>2.54mm 1P-1P 20cm</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
           <t>排</t>
         </is>
       </c>
-      <c r="F24" s="11" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>C895920</t>
         </is>
       </c>
-      <c r="G24" s="12" t="inlineStr">
+      <c r="G26" s="7" t="inlineStr">
         <is>
           <t>¥3</t>
         </is>
       </c>
-      <c r="H24" s="12" t="inlineStr">
+      <c r="H26" s="7" t="inlineStr">
         <is>
           <t>传感器模块 ↔ NUCLEO 引脚连接</t>
         </is>
       </c>
-      <c r="I24" s="12" t="inlineStr">
+      <c r="I26" s="7" t="inlineStr">
         <is>
           <t>10根/排</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>杜邦线 公对公 20cm</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C27" s="11" t="inlineStr">
         <is>
           <t>2.54mm 1P-1P 20cm</t>
         </is>
       </c>
-      <c r="D25" s="6" t="n">
+      <c r="D27" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E25" s="8" t="inlineStr">
+      <c r="E27" s="13" t="inlineStr">
         <is>
           <t>排</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="F27" s="11" t="inlineStr">
         <is>
           <t>C895919</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="G27" s="12" t="inlineStr">
         <is>
           <t>¥3</t>
         </is>
       </c>
-      <c r="H25" s="7" t="inlineStr">
+      <c r="H27" s="12" t="inlineStr">
         <is>
           <t>面包板内跳线</t>
         </is>
       </c>
-      <c r="I25" s="7" t="inlineStr">
+      <c r="I27" s="12" t="inlineStr">
         <is>
           <t>10根/排</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="11" t="n">
-        <v>16</v>
-      </c>
-      <c r="B26" s="12" t="inlineStr">
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>830 孔面包板</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>830 孔 Mini 面包板 165x55mm</t>
         </is>
       </c>
-      <c r="D26" s="11" t="n">
+      <c r="D28" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E26" s="13" t="inlineStr">
+      <c r="E28" s="8" t="inlineStr">
         <is>
           <t>块</t>
         </is>
       </c>
-      <c r="F26" s="11" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>C124363</t>
         </is>
       </c>
-      <c r="G26" s="12" t="inlineStr">
+      <c r="G28" s="7" t="inlineStr">
         <is>
           <t>¥8</t>
         </is>
       </c>
-      <c r="H26" s="12" t="inlineStr">
+      <c r="H28" s="7" t="inlineStr">
         <is>
           <t>模块临时搭接验证</t>
         </is>
       </c>
-      <c r="I26" s="12" t="inlineStr"/>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="6" t="n">
-        <v>17</v>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="I28" s="7" t="inlineStr"/>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="11" t="n">
+        <v>18</v>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>尼龙扎带 3x100mm</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr">
         <is>
           <t>3x100mm 黑色</t>
         </is>
       </c>
-      <c r="D27" s="6" t="n">
+      <c r="D29" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E27" s="8" t="inlineStr">
+      <c r="E29" s="13" t="inlineStr">
         <is>
           <t>包</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="F29" s="11" t="inlineStr">
         <is>
           <t>C306488</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr">
+      <c r="G29" s="12" t="inlineStr">
         <is>
           <t>¥5</t>
         </is>
       </c>
-      <c r="H27" s="7" t="inlineStr">
+      <c r="H29" s="12" t="inlineStr">
         <is>
           <t>固定电池和模块到开发板</t>
         </is>
       </c>
-      <c r="I27" s="7" t="inlineStr">
+      <c r="I29" s="12" t="inlineStr">
         <is>
           <t>100根/包</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="11" t="n">
-        <v>18</v>
-      </c>
-      <c r="B28" s="12" t="inlineStr">
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>热缩管套装</t>
         </is>
       </c>
-      <c r="C28" s="11" t="inlineStr">
+      <c r="C30" s="6" t="inlineStr">
         <is>
           <t>φ1.5/3/5mm 混装</t>
         </is>
       </c>
-      <c r="D28" s="11" t="n">
+      <c r="D30" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E28" s="13" t="inlineStr">
+      <c r="E30" s="8" t="inlineStr">
         <is>
           <t>包</t>
         </is>
       </c>
-      <c r="F28" s="11" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>C275726</t>
         </is>
       </c>
-      <c r="G28" s="12" t="inlineStr">
+      <c r="G30" s="7" t="inlineStr">
         <is>
           <t>¥6</t>
         </is>
       </c>
-      <c r="H28" s="12" t="inlineStr">
+      <c r="H30" s="7" t="inlineStr">
         <is>
           <t>焊接接头绝缘</t>
         </is>
       </c>
-      <c r="I28" s="12" t="inlineStr"/>
-    </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="14" t="inlineStr">
+      <c r="I30" s="7" t="inlineStr"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="14" t="inlineStr">
         <is>
           <t>费用汇总</t>
         </is>
       </c>
-      <c r="B30" s="15" t="n"/>
-      <c r="C30" s="15" t="n"/>
-      <c r="D30" s="15" t="n"/>
-      <c r="E30" s="15" t="n"/>
-      <c r="F30" s="15" t="n"/>
-      <c r="G30" s="15" t="n"/>
-      <c r="H30" s="15" t="n"/>
-      <c r="I30" s="15" t="n"/>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="16" t="inlineStr">
-        <is>
-          <t>开发板: ¥190 (淘宝/得捷) | 立创可购物料 (不含电池): ¥56 | 电池: ¥15 (淘宝) | 总计 约 ¥261</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="16" t="inlineStr">
-        <is>
-          <t>去掉磁力计和蜂鸣器等可选件: 约 ¥250 即可跑通核心功能</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="14" t="inlineStr">
+      <c r="B32" s="15" t="n"/>
+      <c r="C32" s="15" t="n"/>
+      <c r="D32" s="15" t="n"/>
+      <c r="E32" s="15" t="n"/>
+      <c r="F32" s="15" t="n"/>
+      <c r="G32" s="15" t="n"/>
+      <c r="H32" s="15" t="n"/>
+      <c r="I32" s="15" t="n"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>开发板: ¥190 (淘宝/得捷) | 立创可购物料 (不含电池): ¥74 | 电池: ¥15 (淘宝) | 总计 约 ¥279</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>去掉磁力计和蜂鸣器等可选件: 约 ¥268 即可跑通核心功能</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="14" t="inlineStr">
         <is>
           <t>关键参数</t>
-        </is>
-      </c>
-      <c r="B34" s="15" t="n"/>
-      <c r="C34" s="15" t="n"/>
-      <c r="D34" s="15" t="n"/>
-      <c r="E34" s="15" t="n"/>
-      <c r="F34" s="15" t="n"/>
-      <c r="G34" s="15" t="n"/>
-      <c r="H34" s="15" t="n"/>
-      <c r="I34" s="15" t="n"/>
-    </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="17" t="inlineStr">
-        <is>
-          <t>MCU: STM32U575ZIT6Q | Cortex-M33 + FPv5-SP-D16 | 160MHz | 2MB Flash / 786KB SRAM | LQFP144</t>
-        </is>
-      </c>
-      <c r="B35" s="15" t="n"/>
-      <c r="C35" s="15" t="n"/>
-      <c r="D35" s="15" t="n"/>
-      <c r="E35" s="15" t="n"/>
-      <c r="F35" s="15" t="n"/>
-      <c r="G35" s="15" t="n"/>
-      <c r="H35" s="15" t="n"/>
-      <c r="I35" s="15" t="n"/>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="17" t="inlineStr">
-        <is>
-          <t>IMU: 加速度 ±8g / 陀螺仪 ±2000°/s | 采样率 100Hz | I2C 400kHz | 7-bit 地址 0x68</t>
         </is>
       </c>
       <c r="B36" s="15" t="n"/>
@@ -1522,7 +1550,7 @@
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="17" t="inlineStr">
         <is>
-          <t>AHRS: Mahony 互补滤波器 | 加速度+陀螺仪融合 | 磁力计 yaw 修正可选 (AHRS_USE_MAG=0/1)</t>
+          <t>MCU: STM32U575ZIT6Q | Cortex-M33 + FPv5-SP-D16 | 160MHz | 2MB Flash / 786KB SRAM | LQFP144</t>
         </is>
       </c>
       <c r="B37" s="15" t="n"/>
@@ -1537,7 +1565,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="17" t="inlineStr">
         <is>
-          <t>外设引脚 (NUCLEO): LED=PC7 | 按键=PC13 | USART2=PA2(TX)/PA3(RX) | I2C1=PB8(SCL)/PB9(SDA)</t>
+          <t>IMU: 加速度 ±8g / 陀螺仪 ±2000°/s | 采样率 100Hz | I2C 400kHz | 7-bit 地址 0x68</t>
         </is>
       </c>
       <c r="B38" s="15" t="n"/>
@@ -1552,7 +1580,7 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="17" t="inlineStr">
         <is>
-          <t>跌倒检测: Free-fall (0.6g) → Impact (3g) → Post-impact tilt (&gt;60deg) → 5 帧防抖确认</t>
+          <t>AHRS: Mahony 互补滤波器 | 加速度+陀螺仪融合 | 磁力计 yaw 修正可选 (AHRS_USE_MAG=0/1)</t>
         </is>
       </c>
       <c r="B39" s="15" t="n"/>
@@ -1567,7 +1595,7 @@
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="17" t="inlineStr">
         <is>
-          <t>功耗: STOP 模式目标 &lt; 50μA | IMU 运动中断唤醒 | RTC 定时唤醒 | LPBAM 后台外设</t>
+          <t>外设引脚 (NUCLEO): LED=PC7 | 按键=PC13 | USART2=PA2(TX)/PA3(RX) | I2C1=PB8(SCL)/PB9(SDA)</t>
         </is>
       </c>
       <c r="B40" s="15" t="n"/>
@@ -1582,7 +1610,7 @@
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>编译: arm-none-eabi-gcc + Makefile → build/stm32u5_skeleton.elf/.bin/.hex</t>
+          <t>跌倒检测: Free-fall (0.6g) → Impact (3g) → Post-impact tilt (&gt;60deg) → 5 帧防抖确认</t>
         </is>
       </c>
       <c r="B41" s="15" t="n"/>
@@ -1594,27 +1622,58 @@
       <c r="H41" s="15" t="n"/>
       <c r="I41" s="15" t="n"/>
     </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t>功耗: STOP 模式目标 &lt; 50μA | IMU 运动中断唤醒 | RTC 定时唤醒 | LPBAM 后台外设</t>
+        </is>
+      </c>
+      <c r="B42" s="15" t="n"/>
+      <c r="C42" s="15" t="n"/>
+      <c r="D42" s="15" t="n"/>
+      <c r="E42" s="15" t="n"/>
+      <c r="F42" s="15" t="n"/>
+      <c r="G42" s="15" t="n"/>
+      <c r="H42" s="15" t="n"/>
+      <c r="I42" s="15" t="n"/>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>编译: arm-none-eabi-gcc + Makefile → build/stm32u5_skeleton.elf/.bin/.hex</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="n"/>
+      <c r="C43" s="15" t="n"/>
+      <c r="D43" s="15" t="n"/>
+      <c r="E43" s="15" t="n"/>
+      <c r="F43" s="15" t="n"/>
+      <c r="G43" s="15" t="n"/>
+      <c r="H43" s="15" t="n"/>
+      <c r="I43" s="15" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="20">
     <mergeCell ref="A7:I7"/>
+    <mergeCell ref="A25:I25"/>
     <mergeCell ref="A41:I41"/>
     <mergeCell ref="A37:I37"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A21:I21"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A33:I33"/>
     <mergeCell ref="A5:I5"/>
+    <mergeCell ref="A42:I42"/>
     <mergeCell ref="A32:I32"/>
-    <mergeCell ref="A23:I23"/>
-    <mergeCell ref="A35:I35"/>
     <mergeCell ref="A38:I38"/>
-    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="A43:I43"/>
     <mergeCell ref="A10:I10"/>
     <mergeCell ref="A40:I40"/>
-    <mergeCell ref="A31:I31"/>
     <mergeCell ref="A39:I39"/>
     <mergeCell ref="A34:I34"/>
-    <mergeCell ref="A30:I30"/>
     <mergeCell ref="A36:I36"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A16:I16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: add NTAG215 NFC tags to BOM
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Co-authored-by: multica-agent <github@multica.ai>
</commit_message>
<xml_diff>
--- a/STM32U5_BOM.xlsx
+++ b/STM32U5_BOM.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -818,63 +818,63 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>NFC 标签贴纸</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>NTAG215 空白标签</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>张</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>C2892084</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>¥2</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>NFC 标签，可写入急救信息/设备配置</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>搜索"NTAG215 NFC标签"，13.56MHz 504字节</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>四、告警输出</t>
         </is>
       </c>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
-      <c r="H12" s="10" t="n"/>
-      <c r="I12" s="10" t="n"/>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>微型振动马达</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>1027 扁平偏心轮电机</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>个</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>C2895556</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>¥3</t>
-        </is>
-      </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>跌倒/倾斜触觉告警，PWM 调速</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="inlineStr">
-        <is>
-          <t>需配 NPN 三极管驱动 (如 S8050 C2146)</t>
-        </is>
-      </c>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="n"/>
+      <c r="H13" s="10" t="n"/>
+      <c r="I13" s="10" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="11" t="n">
@@ -882,16 +882,16 @@
       </c>
       <c r="B14" s="12" t="inlineStr">
         <is>
-          <t>NPN 三极管</t>
+          <t>微型振动马达</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>S8050 (TO-92)</t>
+          <t>1027 扁平偏心轮电机</t>
         </is>
       </c>
       <c r="D14" s="11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
@@ -900,20 +900,24 @@
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>C2146</t>
+          <t>C2895556</t>
         </is>
       </c>
       <c r="G14" s="12" t="inlineStr">
         <is>
-          <t>¥0.2</t>
+          <t>¥3</t>
         </is>
       </c>
       <c r="H14" s="12" t="inlineStr">
         <is>
-          <t>驱动振动马达</t>
-        </is>
-      </c>
-      <c r="I14" s="12" t="inlineStr"/>
+          <t>跌倒/倾斜触觉告警，PWM 调速</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>需配 NPN 三极管驱动 (如 S8050 C2146)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -921,16 +925,16 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>直插 RGB LED 共阴</t>
+          <t>NPN 三极管</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>5mm 共阴三色 LED</t>
+          <t>S8050 (TO-92)</t>
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
@@ -939,24 +943,20 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>C965027</t>
+          <t>C2146</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>¥1</t>
+          <t>¥0.2</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>状态指示: 绿(正常) 黄(倾斜) 红(跌倒)</t>
-        </is>
-      </c>
-      <c r="I15" s="7" t="inlineStr">
-        <is>
-          <t>需 3 颗 220Ω 限流电阻</t>
-        </is>
-      </c>
+          <t>驱动振动马达</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="11" t="n">
@@ -964,16 +964,16 @@
       </c>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>直插电阻 220Ω</t>
+          <t>直插 RGB LED 共阴</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>1/4W ±5% 碳膜</t>
+          <t>5mm 共阴三色 LED</t>
         </is>
       </c>
       <c r="D16" s="11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
@@ -982,20 +982,24 @@
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>C17405</t>
+          <t>C965027</t>
         </is>
       </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
-          <t>¥0.1</t>
+          <t>¥1</t>
         </is>
       </c>
       <c r="H16" s="12" t="inlineStr">
         <is>
-          <t>RGB LED 限流</t>
-        </is>
-      </c>
-      <c r="I16" s="12" t="inlineStr"/>
+          <t>状态指示: 绿(正常) 黄(倾斜) 红(跌倒)</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>需 3 颗 220Ω 限流电阻</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -1003,100 +1007,96 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
+          <t>直插电阻 220Ω</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>1/4W ±5% 碳膜</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>C17405</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>¥0.1</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>RGB LED 限流</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
           <t>有源蜂鸣器模块 (可选)</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>3.3V 有源蜂鸣器</t>
         </is>
       </c>
-      <c r="D17" s="6" t="n">
+      <c r="D18" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E18" s="13" t="inlineStr">
         <is>
           <t>个</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F18" s="11" t="inlineStr">
         <is>
           <t>C31955</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr">
+      <c r="G18" s="12" t="inlineStr">
         <is>
           <t>¥2</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
+      <c r="H18" s="12" t="inlineStr">
         <is>
           <t>声音告警辅助</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr">
+      <c r="I18" s="12" t="inlineStr">
         <is>
           <t>搜索"3.3V有源蜂鸣器模块"</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="9" t="inlineStr">
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>五、输入交互</t>
         </is>
       </c>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
-      <c r="H18" s="10" t="n"/>
-      <c r="I18" s="10" t="n"/>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>轻触开关 6x6mm</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="inlineStr">
-        <is>
-          <t>6x6x5mm 四脚轻触</t>
-        </is>
-      </c>
-      <c r="D19" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E19" s="13" t="inlineStr">
-        <is>
-          <t>个</t>
-        </is>
-      </c>
-      <c r="F19" s="11" t="inlineStr">
-        <is>
-          <t>C31892</t>
-        </is>
-      </c>
-      <c r="G19" s="12" t="inlineStr">
-        <is>
-          <t>¥0.3</t>
-        </is>
-      </c>
-      <c r="H19" s="12" t="inlineStr">
-        <is>
-          <t>长按解除告警 + 预留功能按键</t>
-        </is>
-      </c>
-      <c r="I19" s="12" t="inlineStr">
-        <is>
-          <t>配 10kΩ 上拉电阻</t>
-        </is>
-      </c>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
+      <c r="H19" s="10" t="n"/>
+      <c r="I19" s="10" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="6" t="n">
@@ -1104,12 +1104,12 @@
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>直插电阻 10kΩ</t>
+          <t>轻触开关 6x6mm</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>1/4W ±5% 碳膜</t>
+          <t>6x6x5mm 四脚轻触</t>
         </is>
       </c>
       <c r="D20" s="6" t="n">
@@ -1122,78 +1122,78 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
+          <t>C31892</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>¥0.3</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>长按解除告警 + 预留功能按键</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="inlineStr">
+        <is>
+          <t>配 10kΩ 上拉电阻</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>直插电阻 10kΩ</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>1/4W ±5% 碳膜</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
           <t>C17408</t>
         </is>
       </c>
-      <c r="G20" s="7" t="inlineStr">
+      <c r="G21" s="12" t="inlineStr">
         <is>
           <t>¥0.1</t>
         </is>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H21" s="12" t="inlineStr">
         <is>
           <t>按键上拉</t>
         </is>
       </c>
-      <c r="I20" s="7" t="inlineStr"/>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="I21" s="12" t="inlineStr"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>六、电源系统</t>
         </is>
       </c>
-      <c r="B21" s="10" t="n"/>
-      <c r="C21" s="10" t="n"/>
-      <c r="D21" s="10" t="n"/>
-      <c r="E21" s="10" t="n"/>
-      <c r="F21" s="10" t="n"/>
-      <c r="G21" s="10" t="n"/>
-      <c r="H21" s="10" t="n"/>
-      <c r="I21" s="10" t="n"/>
-    </row>
-    <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="11" t="n">
-        <v>12</v>
-      </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>AMS1117-3.3V 稳压模块</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="inlineStr">
-        <is>
-          <t>AMS1117-3.3 降压模块</t>
-        </is>
-      </c>
-      <c r="D22" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="13" t="inlineStr">
-        <is>
-          <t>个</t>
-        </is>
-      </c>
-      <c r="F22" s="11" t="inlineStr">
-        <is>
-          <t>C6186</t>
-        </is>
-      </c>
-      <c r="G22" s="12" t="inlineStr">
-        <is>
-          <t>¥2</t>
-        </is>
-      </c>
-      <c r="H22" s="12" t="inlineStr">
-        <is>
-          <t>电池 3.7V → 3.3V 稳定供电</t>
-        </is>
-      </c>
-      <c r="I22" s="12" t="inlineStr">
-        <is>
-          <t>或直接用 NUCLEO Vin 引脚 (5V)</t>
-        </is>
-      </c>
+      <c r="B22" s="10" t="n"/>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="10" t="n"/>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="10" t="n"/>
+      <c r="G22" s="10" t="n"/>
+      <c r="H22" s="10" t="n"/>
+      <c r="I22" s="10" t="n"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="6" t="n">
@@ -1201,12 +1201,12 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>TP4056 锂电池充电模块</t>
+          <t>AMS1117-3.3V 稳压模块</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>TP4056 Type-C 充电板</t>
+          <t>AMS1117-3.3 降压模块</t>
         </is>
       </c>
       <c r="D23" s="6" t="n">
@@ -1219,22 +1219,22 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>C382139</t>
+          <t>C6186</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>¥3</t>
+          <t>¥2</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>锂电池充电管理，含过充过放保护</t>
+          <t>电池 3.7V → 3.3V 稳定供电</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>搜索"TP4056充电模块 Type-C"</t>
+          <t>或直接用 NUCLEO Vin 引脚 (5V)</t>
         </is>
       </c>
     </row>
@@ -1244,12 +1244,12 @@
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>锂聚合物电池</t>
+          <t>TP4056 锂电池充电模块</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>3.7V 800mAh 502535</t>
+          <t>TP4056 Type-C 充电板</t>
         </is>
       </c>
       <c r="D24" s="11" t="n">
@@ -1257,87 +1257,87 @@
       </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
+          <t>个</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>C382139</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>¥3</t>
+        </is>
+      </c>
+      <c r="H24" s="12" t="inlineStr">
+        <is>
+          <t>锂电池充电管理，含过充过放保护</t>
+        </is>
+      </c>
+      <c r="I24" s="12" t="inlineStr">
+        <is>
+          <t>搜索"TP4056充电模块 Type-C"</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>锂聚合物电池</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>3.7V 800mAh 502535</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
           <t>块</t>
         </is>
       </c>
-      <c r="F24" s="11" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G24" s="12" t="inlineStr">
+      <c r="G25" s="7" t="inlineStr">
         <is>
           <t>¥15</t>
         </is>
       </c>
-      <c r="H24" s="12" t="inlineStr">
+      <c r="H25" s="7" t="inlineStr">
         <is>
           <t>可穿戴独立供电</t>
         </is>
       </c>
-      <c r="I24" s="12" t="inlineStr">
+      <c r="I25" s="7" t="inlineStr">
         <is>
           <t>淘宝购买，立创不售电池</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
         <is>
           <t>七、连接与固定</t>
         </is>
       </c>
-      <c r="B25" s="10" t="n"/>
-      <c r="C25" s="10" t="n"/>
-      <c r="D25" s="10" t="n"/>
-      <c r="E25" s="10" t="n"/>
-      <c r="F25" s="10" t="n"/>
-      <c r="G25" s="10" t="n"/>
-      <c r="H25" s="10" t="n"/>
-      <c r="I25" s="10" t="n"/>
-    </row>
-    <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
-        <is>
-          <t>杜邦线 母对母 20cm</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>2.54mm 1P-1P 20cm</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="8" t="inlineStr">
-        <is>
-          <t>排</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>C895920</t>
-        </is>
-      </c>
-      <c r="G26" s="7" t="inlineStr">
-        <is>
-          <t>¥3</t>
-        </is>
-      </c>
-      <c r="H26" s="7" t="inlineStr">
-        <is>
-          <t>传感器模块 ↔ NUCLEO 引脚连接</t>
-        </is>
-      </c>
-      <c r="I26" s="7" t="inlineStr">
-        <is>
-          <t>10根/排</t>
-        </is>
-      </c>
+      <c r="B26" s="10" t="n"/>
+      <c r="C26" s="10" t="n"/>
+      <c r="D26" s="10" t="n"/>
+      <c r="E26" s="10" t="n"/>
+      <c r="F26" s="10" t="n"/>
+      <c r="G26" s="10" t="n"/>
+      <c r="H26" s="10" t="n"/>
+      <c r="I26" s="10" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="11" t="n">
@@ -1345,7 +1345,7 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>杜邦线 公对公 20cm</t>
+          <t>杜邦线 母对母 20cm</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>C895919</t>
+          <t>C895920</t>
         </is>
       </c>
       <c r="G27" s="12" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="H27" s="12" t="inlineStr">
         <is>
-          <t>面包板内跳线</t>
+          <t>传感器模块 ↔ NUCLEO 引脚连接</t>
         </is>
       </c>
       <c r="I27" s="12" t="inlineStr">
@@ -1388,12 +1388,12 @@
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>830 孔面包板</t>
+          <t>杜邦线 公对公 20cm</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>830 孔 Mini 面包板 165x55mm</t>
+          <t>2.54mm 1P-1P 20cm</t>
         </is>
       </c>
       <c r="D28" s="6" t="n">
@@ -1401,25 +1401,29 @@
       </c>
       <c r="E28" s="8" t="inlineStr">
         <is>
-          <t>块</t>
+          <t>排</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>C124363</t>
+          <t>C895919</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>¥8</t>
+          <t>¥3</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>模块临时搭接验证</t>
-        </is>
-      </c>
-      <c r="I28" s="7" t="inlineStr"/>
+          <t>面包板内跳线</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t>10根/排</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="11" t="n">
@@ -1427,12 +1431,12 @@
       </c>
       <c r="B29" s="12" t="inlineStr">
         <is>
-          <t>尼龙扎带 3x100mm</t>
+          <t>830 孔面包板</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>3x100mm 黑色</t>
+          <t>830 孔 Mini 面包板 165x55mm</t>
         </is>
       </c>
       <c r="D29" s="11" t="n">
@@ -1440,29 +1444,25 @@
       </c>
       <c r="E29" s="13" t="inlineStr">
         <is>
-          <t>包</t>
+          <t>块</t>
         </is>
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>C306488</t>
+          <t>C124363</t>
         </is>
       </c>
       <c r="G29" s="12" t="inlineStr">
         <is>
-          <t>¥5</t>
+          <t>¥8</t>
         </is>
       </c>
       <c r="H29" s="12" t="inlineStr">
         <is>
-          <t>固定电池和模块到开发板</t>
-        </is>
-      </c>
-      <c r="I29" s="12" t="inlineStr">
-        <is>
-          <t>100根/包</t>
-        </is>
-      </c>
+          <t>模块临时搭接验证</t>
+        </is>
+      </c>
+      <c r="I29" s="12" t="inlineStr"/>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="6" t="n">
@@ -1470,12 +1470,12 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>热缩管套装</t>
+          <t>尼龙扎带 3x100mm</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>φ1.5/3/5mm 混装</t>
+          <t>3x100mm 黑色</t>
         </is>
       </c>
       <c r="D30" s="6" t="n">
@@ -1488,69 +1488,97 @@
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
+          <t>C306488</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>¥5</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>固定电池和模块到开发板</t>
+        </is>
+      </c>
+      <c r="I30" s="7" t="inlineStr">
+        <is>
+          <t>100根/包</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>热缩管套装</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>φ1.5/3/5mm 混装</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>包</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
           <t>C275726</t>
         </is>
       </c>
-      <c r="G30" s="7" t="inlineStr">
+      <c r="G31" s="12" t="inlineStr">
         <is>
           <t>¥6</t>
         </is>
       </c>
-      <c r="H30" s="7" t="inlineStr">
+      <c r="H31" s="12" t="inlineStr">
         <is>
           <t>焊接接头绝缘</t>
         </is>
       </c>
-      <c r="I30" s="7" t="inlineStr"/>
-    </row>
-    <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="14" t="inlineStr">
+      <c r="I31" s="12" t="inlineStr"/>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="14" t="inlineStr">
         <is>
           <t>费用汇总</t>
         </is>
       </c>
-      <c r="B32" s="15" t="n"/>
-      <c r="C32" s="15" t="n"/>
-      <c r="D32" s="15" t="n"/>
-      <c r="E32" s="15" t="n"/>
-      <c r="F32" s="15" t="n"/>
-      <c r="G32" s="15" t="n"/>
-      <c r="H32" s="15" t="n"/>
-      <c r="I32" s="15" t="n"/>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="16" t="inlineStr">
-        <is>
-          <t>开发板: ¥190 (淘宝/得捷) | 立创可购物料 (不含电池): ¥74 | 电池: ¥15 (淘宝) | 总计 约 ¥279</t>
-        </is>
-      </c>
+      <c r="B33" s="15" t="n"/>
+      <c r="C33" s="15" t="n"/>
+      <c r="D33" s="15" t="n"/>
+      <c r="E33" s="15" t="n"/>
+      <c r="F33" s="15" t="n"/>
+      <c r="G33" s="15" t="n"/>
+      <c r="H33" s="15" t="n"/>
+      <c r="I33" s="15" t="n"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="16" t="inlineStr">
         <is>
-          <t>去掉磁力计和蜂鸣器等可选件: 约 ¥268 即可跑通核心功能</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="22" customHeight="1">
-      <c r="A36" s="14" t="inlineStr">
+          <t>开发板: ¥190 (淘宝/得捷) | 立创可购物料 (不含电池): ¥84 | 电池: ¥15 (淘宝) | 总计 约 ¥289</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>去掉磁力计和蜂鸣器等可选件: 约 ¥276 即可跑通核心功能</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="14" t="inlineStr">
         <is>
           <t>关键参数</t>
-        </is>
-      </c>
-      <c r="B36" s="15" t="n"/>
-      <c r="C36" s="15" t="n"/>
-      <c r="D36" s="15" t="n"/>
-      <c r="E36" s="15" t="n"/>
-      <c r="F36" s="15" t="n"/>
-      <c r="G36" s="15" t="n"/>
-      <c r="H36" s="15" t="n"/>
-      <c r="I36" s="15" t="n"/>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="17" t="inlineStr">
-        <is>
-          <t>MCU: STM32U575ZIT6Q | Cortex-M33 + FPv5-SP-D16 | 160MHz | 2MB Flash / 786KB SRAM | LQFP144</t>
         </is>
       </c>
       <c r="B37" s="15" t="n"/>
@@ -1565,7 +1593,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="17" t="inlineStr">
         <is>
-          <t>IMU: 加速度 ±8g / 陀螺仪 ±2000°/s | 采样率 100Hz | I2C 400kHz | 7-bit 地址 0x68</t>
+          <t>MCU: STM32U575ZIT6Q | Cortex-M33 + FPv5-SP-D16 | 160MHz | 2MB Flash / 786KB SRAM | LQFP144</t>
         </is>
       </c>
       <c r="B38" s="15" t="n"/>
@@ -1580,7 +1608,7 @@
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="17" t="inlineStr">
         <is>
-          <t>AHRS: Mahony 互补滤波器 | 加速度+陀螺仪融合 | 磁力计 yaw 修正可选 (AHRS_USE_MAG=0/1)</t>
+          <t>IMU: 加速度 ±8g / 陀螺仪 ±2000°/s | 采样率 100Hz | I2C 400kHz | 7-bit 地址 0x68</t>
         </is>
       </c>
       <c r="B39" s="15" t="n"/>
@@ -1595,7 +1623,7 @@
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="17" t="inlineStr">
         <is>
-          <t>外设引脚 (NUCLEO): LED=PC7 | 按键=PC13 | USART2=PA2(TX)/PA3(RX) | I2C1=PB8(SCL)/PB9(SDA)</t>
+          <t>AHRS: Mahony 互补滤波器 | 加速度+陀螺仪融合 | 磁力计 yaw 修正可选 (AHRS_USE_MAG=0/1)</t>
         </is>
       </c>
       <c r="B40" s="15" t="n"/>
@@ -1610,7 +1638,7 @@
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
-          <t>跌倒检测: Free-fall (0.6g) → Impact (3g) → Post-impact tilt (&gt;60deg) → 5 帧防抖确认</t>
+          <t>外设引脚 (NUCLEO): LED=PC7 | 按键=PC13 | USART2=PA2(TX)/PA3(RX) | I2C1=PB8(SCL)/PB9(SDA)</t>
         </is>
       </c>
       <c r="B41" s="15" t="n"/>
@@ -1625,7 +1653,7 @@
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="17" t="inlineStr">
         <is>
-          <t>功耗: STOP 模式目标 &lt; 50μA | IMU 运动中断唤醒 | RTC 定时唤醒 | LPBAM 后台外设</t>
+          <t>跌倒检测: Free-fall (0.6g) → Impact (3g) → Post-impact tilt (&gt;60deg) → 5 帧防抖确认</t>
         </is>
       </c>
       <c r="B42" s="15" t="n"/>
@@ -1640,7 +1668,7 @@
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="17" t="inlineStr">
         <is>
-          <t>编译: arm-none-eabi-gcc + Makefile → build/stm32u5_skeleton.elf/.bin/.hex</t>
+          <t>功耗: STOP 模式目标 &lt; 50μA | IMU 运动中断唤醒 | RTC 定时唤醒 | LPBAM 后台外设</t>
         </is>
       </c>
       <c r="B43" s="15" t="n"/>
@@ -1652,27 +1680,42 @@
       <c r="H43" s="15" t="n"/>
       <c r="I43" s="15" t="n"/>
     </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t>编译: arm-none-eabi-gcc + Makefile → build/stm32u5_skeleton.elf/.bin/.hex</t>
+        </is>
+      </c>
+      <c r="B44" s="15" t="n"/>
+      <c r="C44" s="15" t="n"/>
+      <c r="D44" s="15" t="n"/>
+      <c r="E44" s="15" t="n"/>
+      <c r="F44" s="15" t="n"/>
+      <c r="G44" s="15" t="n"/>
+      <c r="H44" s="15" t="n"/>
+      <c r="I44" s="15" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="20">
     <mergeCell ref="A7:I7"/>
-    <mergeCell ref="A25:I25"/>
     <mergeCell ref="A41:I41"/>
     <mergeCell ref="A37:I37"/>
-    <mergeCell ref="A18:I18"/>
-    <mergeCell ref="A12:I12"/>
-    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="A26:I26"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A33:I33"/>
     <mergeCell ref="A5:I5"/>
     <mergeCell ref="A42:I42"/>
-    <mergeCell ref="A32:I32"/>
+    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="A35:I35"/>
     <mergeCell ref="A38:I38"/>
     <mergeCell ref="A43:I43"/>
+    <mergeCell ref="A19:I19"/>
     <mergeCell ref="A10:I10"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A44:I44"/>
     <mergeCell ref="A40:I40"/>
     <mergeCell ref="A39:I39"/>
     <mergeCell ref="A34:I34"/>
-    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>